<commit_message>
- connects scale LCDs directly to scale 1 and 2 - adds support for Schuilenburg machines equipped with Unitronics PLC - adds ALT/OPTION click on template name to toggle event replay - adds notification message if schedule fails to load template - pushes version
</commit_message>
<xml_diff>
--- a/doc/help_dialogs/Input_files/keyboardshortcuts.xlsx
+++ b/doc/help_dialogs/Input_files/keyboardshortcuts.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Keyboard Shortcuts" sheetId="1" state="visible" r:id="rId3"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="244">
   <si>
     <t xml:space="preserve">KEYBOARD SHORTCUTS</t>
   </si>
@@ -155,12 +155,6 @@
     <t xml:space="preserve">Toggle PID mode</t>
   </si>
   <si>
-    <t xml:space="preserve">J</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Toggle Playback Events</t>
-  </si>
-  <si>
     <t xml:space="preserve">H\nCTRL+H [Win]</t>
   </si>
   <si>
@@ -292,6 +286,37 @@
   </si>
   <si>
     <t xml:space="preserve">Only when a Background profile is loaded</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">OPTION click on Background Profile Title </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> [Mac]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">\nALT click on Background Profile Title [Win]</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Toggle Playback Events</t>
   </si>
   <si>
     <t xml:space="preserve">Double click on Graph canvas</t>
@@ -779,7 +804,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -815,6 +840,11 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <i val="true"/>
@@ -911,7 +941,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -919,7 +949,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1047,7 +1077,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B35"/>
+  <dimension ref="A1:B1048576"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="33.54"/>
@@ -1227,11 +1257,11 @@
         <v>42</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="s">
+    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="1" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1259,15 +1289,15 @@
         <v>50</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="22.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" s="3" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="22.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="33.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
         <v>53</v>
       </c>
@@ -1275,8 +1305,8 @@
         <v>54</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="33.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="2" t="s">
+    <row r="29" customFormat="false" ht="22.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="4" t="s">
         <v>55</v>
       </c>
       <c r="B29" s="3" t="s">
@@ -1291,11 +1321,11 @@
         <v>58</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="22.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4" t="s">
+    <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B31" s="3" t="s">
+      <c r="B31" s="1" t="s">
         <v>60</v>
       </c>
     </row>
@@ -1323,14 +1353,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>68</v>
-      </c>
-    </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1347,7 +1370,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D50"/>
+  <dimension ref="A1:D51"/>
   <sheetFormatPr defaultColWidth="9.18359375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="5" width="53"/>
@@ -1359,240 +1382,240 @@
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="D2" s="5" t="s">
         <v>71</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="D3" s="5" t="s">
         <v>75</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>78</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="D5" s="5" t="s">
         <v>81</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="C6" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="D6" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="C6" s="5" t="s">
+    </row>
+    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="B7" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="22.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
+      <c r="D7" s="5" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="22.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="B7" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="C7" s="7" t="s">
+      <c r="B8" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C8" s="7" t="s">
         <v>89</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>98</v>
+        <v>95</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C18" s="5" t="s">
         <v>110</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>115</v>
+        <v>110</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1600,13 +1623,13 @@
         <v>116</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1614,110 +1637,110 @@
         <v>116</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>124</v>
+        <v>77</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>127</v>
+        <v>77</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>132</v>
+        <v>77</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>133</v>
+        <v>123</v>
       </c>
       <c r="B27" s="5" t="s">
         <v>131</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B28" s="5" t="s">
         <v>131</v>
       </c>
       <c r="C28" s="1" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="C29" s="1" t="s">
         <v>136</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="22.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="B29" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="D29" s="7" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="22.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="B30" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="D30" s="7" t="s">
         <v>140</v>
@@ -1725,13 +1748,13 @@
     </row>
     <row r="31" customFormat="false" ht="22.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B31" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D31" s="7" t="s">
         <v>140</v>
@@ -1739,113 +1762,113 @@
     </row>
     <row r="32" customFormat="false" ht="22.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B32" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C32" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="D32" s="7" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="22.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="C33" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="D32" s="7" t="s">
+      <c r="D33" s="7" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="22.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="8" t="s">
+    <row r="34" customFormat="false" ht="22.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="B33" s="7" t="s">
+      <c r="B34" s="7" t="s">
         <v>149</v>
       </c>
-      <c r="C33" s="5" t="s">
+      <c r="C34" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="D33" s="5" t="s">
+      <c r="D34" s="5" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="8" t="s">
+    <row r="35" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="8" t="s">
         <v>152</v>
-      </c>
-      <c r="B34" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="C34" s="5" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="22.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="6" t="s">
-        <v>155</v>
       </c>
       <c r="B35" s="7" t="s">
         <v>153</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="22.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="B36" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="22.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="B36" s="7" t="s">
+      <c r="B37" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="C36" s="5" t="s">
+      <c r="C37" s="5" t="s">
         <v>159</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="6" t="s">
-        <v>160</v>
-      </c>
-      <c r="B37" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="C37" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="D37" s="5" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="6" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="B38" s="5" t="s">
         <v>161</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>165</v>
+        <v>162</v>
+      </c>
+      <c r="D38" s="5" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="6" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B39" s="5" t="s">
         <v>161</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="D39" s="5" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="6" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="B40" s="5" t="s">
         <v>161</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D40" s="5" t="s">
         <v>168</v>
@@ -1853,13 +1876,13 @@
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="6" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B41" s="5" t="s">
         <v>161</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D41" s="5" t="s">
         <v>168</v>
@@ -1867,13 +1890,13 @@
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="6" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>174</v>
+        <v>161</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="D42" s="5" t="s">
         <v>168</v>
@@ -1884,10 +1907,10 @@
         <v>173</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D43" s="5" t="s">
         <v>168</v>
@@ -1895,60 +1918,63 @@
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="6" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>180</v>
+        <v>177</v>
+      </c>
+      <c r="D44" s="5" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="6" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="B46" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="C46" s="5" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="6" t="s">
         <v>184</v>
       </c>
-      <c r="B46" s="5" t="s">
+      <c r="B47" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="C46" s="5" t="s">
+      <c r="C47" s="5" t="s">
         <v>186</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="B47" s="5" t="s">
-        <v>188</v>
-      </c>
-      <c r="C47" s="5" t="s">
-        <v>189</v>
-      </c>
-      <c r="D47" s="5" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>193</v>
+        <v>189</v>
+      </c>
+      <c r="D48" s="5" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1956,10 +1982,10 @@
         <v>191</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1967,9 +1993,20 @@
         <v>191</v>
       </c>
       <c r="B50" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="C50" s="5" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="B51" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="C50" s="5" t="s">
+      <c r="C51" s="5" t="s">
         <v>197</v>
       </c>
     </row>
@@ -2010,7 +2047,7 @@
         <v>199</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2227,7 +2264,7 @@
         <v>242</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C22" s="11" t="s">
         <v>243</v>

</xml_diff>